<commit_message>
Removed non_text_columns list as the format can simply be set directly in excel and pandas seem to respect it sufficiently.
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://steelcase-my.sharepoint.com/personal/ladam_steelcase_com/Documents/SAP/Scripts/python/octopus2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{0618BC03-5275-40B5-9B57-AB5B30C27A46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CAF9D29A-D039-4BAF-98CD-0242640E9613}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="13_ncr:1_{0618BC03-5275-40B5-9B57-AB5B30C27A46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CEAA041-D201-4FA6-83FB-FD11AF656351}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="33">
   <si>
     <t>Material</t>
   </si>
@@ -134,6 +134,9 @@
   </si>
   <si>
     <t>0.01</t>
+  </si>
+  <si>
+    <t>0001</t>
   </si>
 </sst>
 </file>
@@ -177,12 +180,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -467,13 +471,14 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -493,8 +498,8 @@
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
-        <v>3</v>
+      <c r="B2" s="2" t="s">
+        <v>32</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -510,7 +515,7 @@
       <c r="A3" t="s">
         <v>20</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C3" t="s">
@@ -527,7 +532,7 @@
       <c r="A4" t="s">
         <v>20</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C4" t="s">
@@ -544,7 +549,7 @@
       <c r="A5" t="s">
         <v>2</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C5" t="s">
@@ -561,7 +566,7 @@
       <c r="A6" t="s">
         <v>2</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C6" t="s">
@@ -578,7 +583,7 @@
       <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C7" t="s">
@@ -595,7 +600,7 @@
       <c r="A8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C8" t="s">
@@ -612,7 +617,7 @@
       <c r="A9" t="s">
         <v>11</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C9" t="s">
@@ -629,7 +634,7 @@
       <c r="A10" t="s">
         <v>11</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C10" t="s">
@@ -646,7 +651,7 @@
       <c r="A11" t="s">
         <v>2</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C11" t="s">
@@ -666,7 +671,7 @@
       <c r="A12" t="s">
         <v>2</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C12" t="s">

</xml_diff>

<commit_message>
added option to input file/settings to read all data as text which is still needed because pandas still converts 001 to 1 if all values in that column are numeric! Also corrected a bug - init task was always executed.
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://steelcase-my.sharepoint.com/personal/ladam_steelcase_com/Documents/SAP/Scripts/python/octopus2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="13_ncr:1_{0618BC03-5275-40B5-9B57-AB5B30C27A46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CEAA041-D201-4FA6-83FB-FD11AF656351}"/>
+  <xr:revisionPtr revIDLastSave="74" documentId="13_ncr:1_{0618BC03-5275-40B5-9B57-AB5B30C27A46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE58DA2D-2ABF-4BDA-B089-6369F523D34B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="34">
   <si>
     <t>Material</t>
   </si>
@@ -118,15 +118,9 @@
     <t>can live here</t>
   </si>
   <si>
-    <t>Non_text_columns</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
-    <t>Date,</t>
-  </si>
-  <si>
     <t>Number</t>
   </si>
   <si>
@@ -137,6 +131,15 @@
   </si>
   <si>
     <t>0001</t>
+  </si>
+  <si>
+    <t>Read all columns as text</t>
+  </si>
+  <si>
+    <t>All columns of input file are read as text. [yes/no]</t>
+  </si>
+  <si>
+    <t>no</t>
   </si>
 </sst>
 </file>
@@ -488,10 +491,10 @@
         <v>13</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -499,7 +502,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
         <v>8</v>
@@ -610,7 +613,7 @@
         <v>46188</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -627,7 +630,7 @@
         <v>46189</v>
       </c>
       <c r="F9" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -697,7 +700,7 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="97.28515625" bestFit="1" customWidth="1"/>
   </cols>
@@ -715,12 +718,14 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="C2" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">

</xml_diff>